<commit_message>
endo of exposure testing for now: no significant change from transaction cost changes
</commit_message>
<xml_diff>
--- a/Selected Strategy mode/results/batchruns/batch_selected_config_strategy.xlsx
+++ b/Selected Strategy mode/results/batchruns/batch_selected_config_strategy.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="61" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="366" uniqueCount="60">
   <si>
     <t>Ticker</t>
   </si>
@@ -494,37 +494,37 @@
         <v>339.63177562489244</v>
       </c>
       <c r="J2" s="0">
-        <v>432.28680471328511</v>
+        <v>418.61112781662274</v>
       </c>
       <c r="K2" s="0">
-        <v>419.30612603563463</v>
+        <v>404.55630860215217</v>
       </c>
       <c r="L2" s="0">
-        <v>432.28680471328511</v>
+        <v>418.61112781662274</v>
       </c>
       <c r="M2" s="0">
         <v>-33.715385820778607</v>
       </c>
       <c r="N2" s="0">
-        <v>-24.073604766594158</v>
+        <v>-24.373627988709799</v>
       </c>
       <c r="O2" s="0">
-        <v>-24.497326364091077</v>
+        <v>-24.797283106279878</v>
       </c>
       <c r="P2" s="0">
-        <v>-24.073604766594158</v>
+        <v>-24.373627988709799</v>
       </c>
       <c r="Q2" s="0">
         <v>0.82591294677085225</v>
       </c>
       <c r="R2" s="0">
-        <v>1.0279386507973149</v>
+        <v>1.0130118248433477</v>
       </c>
       <c r="S2" s="0">
-        <v>1.017688926866156</v>
+        <v>1.0011427955385548</v>
       </c>
       <c r="T2" s="0">
-        <v>1.0279386507973149</v>
+        <v>1.0130118248433477</v>
       </c>
       <c r="U2" s="0">
         <v>1</v>
@@ -599,37 +599,37 @@
         <v>0</v>
       </c>
       <c r="AS2" s="0">
-        <v>92.655029088392652</v>
+        <v>78.979352191730271</v>
       </c>
       <c r="AT2" s="0">
-        <v>79.674350410742178</v>
+        <v>64.92453297725973</v>
       </c>
       <c r="AU2" s="0">
-        <v>92.655029088392652</v>
+        <v>78.979352191730271</v>
       </c>
       <c r="AV2" s="0">
         <v>0</v>
       </c>
       <c r="AW2" s="0">
-        <v>9.6417810541844506</v>
+        <v>9.3417578320688079</v>
       </c>
       <c r="AX2" s="0">
-        <v>9.2180594566875325</v>
+        <v>8.9181027144987333</v>
       </c>
       <c r="AY2" s="0">
-        <v>9.6417810541844506</v>
+        <v>9.3417578320688079</v>
       </c>
       <c r="AZ2" s="0">
         <v>0</v>
       </c>
       <c r="BA2" s="0">
-        <v>0.20202570402646269</v>
+        <v>0.18709887807249548</v>
       </c>
       <c r="BB2" s="0">
-        <v>0.19177598009530372</v>
+        <v>0.17522984876770253</v>
       </c>
       <c r="BC2" s="0">
-        <v>0.20202570402646269</v>
+        <v>0.18709887807249548</v>
       </c>
     </row>
     <row r="3">
@@ -661,37 +661,37 @@
         <v>676.99257536452114</v>
       </c>
       <c r="J3" s="0">
-        <v>719.03877011519592</v>
+        <v>688.45854647972556</v>
       </c>
       <c r="K3" s="0">
-        <v>722.77091668471223</v>
+        <v>690.11412086924599</v>
       </c>
       <c r="L3" s="0">
-        <v>722.77091668471223</v>
+        <v>690.11412086924599</v>
       </c>
       <c r="M3" s="0">
         <v>-35.119666881826539</v>
       </c>
       <c r="N3" s="0">
-        <v>-30.159087754807157</v>
+        <v>-30.715404023167391</v>
       </c>
       <c r="O3" s="0">
-        <v>-30.150321939563472</v>
+        <v>-31.180228856880031</v>
       </c>
       <c r="P3" s="0">
-        <v>-30.150321939563472</v>
+        <v>-31.180228856880031</v>
       </c>
       <c r="Q3" s="0">
         <v>0.93436024338566648</v>
       </c>
       <c r="R3" s="0">
-        <v>1.0483454895318489</v>
+        <v>1.0309865137384657</v>
       </c>
       <c r="S3" s="0">
-        <v>1.0542780345112299</v>
+        <v>1.0356178158091829</v>
       </c>
       <c r="T3" s="0">
-        <v>1.0542780345112299</v>
+        <v>1.0356178158091829</v>
       </c>
       <c r="U3" s="0">
         <v>1</v>
@@ -766,37 +766,37 @@
         <v>0</v>
       </c>
       <c r="AS3" s="0">
-        <v>42.046194750674815</v>
+        <v>11.465971115204443</v>
       </c>
       <c r="AT3" s="0">
-        <v>45.778341320191096</v>
+        <v>13.121545504724885</v>
       </c>
       <c r="AU3" s="0">
-        <v>45.778341320191096</v>
+        <v>13.121545504724885</v>
       </c>
       <c r="AV3" s="0">
         <v>0</v>
       </c>
       <c r="AW3" s="0">
-        <v>4.9605791270193826</v>
+        <v>4.4042628586591466</v>
       </c>
       <c r="AX3" s="0">
-        <v>4.9693449422630653</v>
+        <v>3.9394380249465066</v>
       </c>
       <c r="AY3" s="0">
-        <v>4.9693449422630653</v>
+        <v>3.9394380249465066</v>
       </c>
       <c r="AZ3" s="0">
         <v>0</v>
       </c>
       <c r="BA3" s="0">
-        <v>0.11398524614618244</v>
+        <v>0.096626270352799248</v>
       </c>
       <c r="BB3" s="0">
-        <v>0.11991779112556344</v>
+        <v>0.10125757242351641</v>
       </c>
       <c r="BC3" s="0">
-        <v>0.11991779112556344</v>
+        <v>0.10125757242351641</v>
       </c>
     </row>
     <row r="4">
@@ -828,37 +828,37 @@
         <v>456.72653958944289</v>
       </c>
       <c r="J4" s="0">
-        <v>557.19483979185463</v>
+        <v>540.20486815260654</v>
       </c>
       <c r="K4" s="0">
-        <v>570.06668567619192</v>
+        <v>549.89140858672499</v>
       </c>
       <c r="L4" s="0">
-        <v>570.06668567619192</v>
+        <v>549.89140858672499</v>
       </c>
       <c r="M4" s="0">
         <v>-32.676170186531131</v>
       </c>
       <c r="N4" s="0">
-        <v>-30.391654756053587</v>
+        <v>-30.951141600791221</v>
       </c>
       <c r="O4" s="0">
-        <v>-29.871419929998801</v>
+        <v>-30.433364581043254</v>
       </c>
       <c r="P4" s="0">
-        <v>-29.871419929998801</v>
+        <v>-30.433364581043254</v>
       </c>
       <c r="Q4" s="0">
         <v>0.85109775601218884</v>
       </c>
       <c r="R4" s="0">
-        <v>1.0282651002659589</v>
+        <v>1.0146928311762144</v>
       </c>
       <c r="S4" s="0">
-        <v>1.0422206316925515</v>
+        <v>1.0264096419169355</v>
       </c>
       <c r="T4" s="0">
-        <v>1.0422206316925515</v>
+        <v>1.0264096419169355</v>
       </c>
       <c r="U4" s="0">
         <v>1</v>
@@ -933,37 +933,37 @@
         <v>0</v>
       </c>
       <c r="AS4" s="0">
-        <v>100.46830020241168</v>
+        <v>83.478328563163643</v>
       </c>
       <c r="AT4" s="0">
-        <v>113.340146086749</v>
+        <v>93.164868997282113</v>
       </c>
       <c r="AU4" s="0">
-        <v>113.340146086749</v>
+        <v>93.164868997282113</v>
       </c>
       <c r="AV4" s="0">
         <v>0</v>
       </c>
       <c r="AW4" s="0">
-        <v>2.2845154304775406</v>
+        <v>1.7250285857399072</v>
       </c>
       <c r="AX4" s="0">
-        <v>2.804750256532329</v>
+        <v>2.2428056054878742</v>
       </c>
       <c r="AY4" s="0">
-        <v>2.804750256532329</v>
+        <v>2.2428056054878742</v>
       </c>
       <c r="AZ4" s="0">
         <v>0</v>
       </c>
       <c r="BA4" s="0">
-        <v>0.17716734425377001</v>
+        <v>0.16359507516402561</v>
       </c>
       <c r="BB4" s="0">
-        <v>0.19112287568036268</v>
+        <v>0.17531188590474667</v>
       </c>
       <c r="BC4" s="0">
-        <v>0.19112287568036268</v>
+        <v>0.17531188590474667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new model: soft regime filter
</commit_message>
<xml_diff>
--- a/Selected Strategy mode/results/batchruns/batch_selected_config_strategy.xlsx
+++ b/Selected Strategy mode/results/batchruns/batch_selected_config_strategy.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="366" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="1216" uniqueCount="60">
   <si>
     <t>Ticker</t>
   </si>
@@ -494,37 +494,37 @@
         <v>339.63177562489244</v>
       </c>
       <c r="J2" s="0">
-        <v>418.61112781662274</v>
+        <v>432.28680471328511</v>
       </c>
       <c r="K2" s="0">
-        <v>404.55630860215217</v>
+        <v>419.30612603563463</v>
       </c>
       <c r="L2" s="0">
-        <v>418.61112781662274</v>
+        <v>432.28680471328511</v>
       </c>
       <c r="M2" s="0">
         <v>-33.715385820778607</v>
       </c>
       <c r="N2" s="0">
-        <v>-24.373627988709799</v>
+        <v>-24.073604766594158</v>
       </c>
       <c r="O2" s="0">
-        <v>-24.797283106279878</v>
+        <v>-24.497326364091077</v>
       </c>
       <c r="P2" s="0">
-        <v>-24.373627988709799</v>
+        <v>-24.073604766594158</v>
       </c>
       <c r="Q2" s="0">
         <v>0.82591294677085225</v>
       </c>
       <c r="R2" s="0">
-        <v>1.0130118248433477</v>
+        <v>1.0279386507973149</v>
       </c>
       <c r="S2" s="0">
-        <v>1.0011427955385548</v>
+        <v>1.017688926866156</v>
       </c>
       <c r="T2" s="0">
-        <v>1.0130118248433477</v>
+        <v>1.0279386507973149</v>
       </c>
       <c r="U2" s="0">
         <v>1</v>
@@ -599,37 +599,37 @@
         <v>0</v>
       </c>
       <c r="AS2" s="0">
-        <v>78.979352191730271</v>
+        <v>92.655029088392652</v>
       </c>
       <c r="AT2" s="0">
-        <v>64.92453297725973</v>
+        <v>79.674350410742178</v>
       </c>
       <c r="AU2" s="0">
-        <v>78.979352191730271</v>
+        <v>92.655029088392652</v>
       </c>
       <c r="AV2" s="0">
         <v>0</v>
       </c>
       <c r="AW2" s="0">
-        <v>9.3417578320688079</v>
+        <v>9.6417810541844506</v>
       </c>
       <c r="AX2" s="0">
-        <v>8.9181027144987333</v>
+        <v>9.2180594566875325</v>
       </c>
       <c r="AY2" s="0">
-        <v>9.3417578320688079</v>
+        <v>9.6417810541844506</v>
       </c>
       <c r="AZ2" s="0">
         <v>0</v>
       </c>
       <c r="BA2" s="0">
-        <v>0.18709887807249548</v>
+        <v>0.20202570402646269</v>
       </c>
       <c r="BB2" s="0">
-        <v>0.17522984876770253</v>
+        <v>0.19177598009530372</v>
       </c>
       <c r="BC2" s="0">
-        <v>0.18709887807249548</v>
+        <v>0.20202570402646269</v>
       </c>
     </row>
     <row r="3">
@@ -661,37 +661,37 @@
         <v>676.99257536452114</v>
       </c>
       <c r="J3" s="0">
-        <v>688.45854647972556</v>
+        <v>719.03877011519592</v>
       </c>
       <c r="K3" s="0">
-        <v>690.11412086924599</v>
+        <v>722.77091668471223</v>
       </c>
       <c r="L3" s="0">
-        <v>690.11412086924599</v>
+        <v>722.77091668471223</v>
       </c>
       <c r="M3" s="0">
         <v>-35.119666881826539</v>
       </c>
       <c r="N3" s="0">
-        <v>-30.715404023167391</v>
+        <v>-30.159087754807157</v>
       </c>
       <c r="O3" s="0">
-        <v>-31.180228856880031</v>
+        <v>-30.150321939563472</v>
       </c>
       <c r="P3" s="0">
-        <v>-31.180228856880031</v>
+        <v>-30.150321939563472</v>
       </c>
       <c r="Q3" s="0">
         <v>0.93436024338566648</v>
       </c>
       <c r="R3" s="0">
-        <v>1.0309865137384657</v>
+        <v>1.0483454895318489</v>
       </c>
       <c r="S3" s="0">
-        <v>1.0356178158091829</v>
+        <v>1.0542780345112299</v>
       </c>
       <c r="T3" s="0">
-        <v>1.0356178158091829</v>
+        <v>1.0542780345112299</v>
       </c>
       <c r="U3" s="0">
         <v>1</v>
@@ -766,37 +766,37 @@
         <v>0</v>
       </c>
       <c r="AS3" s="0">
-        <v>11.465971115204443</v>
+        <v>42.046194750674815</v>
       </c>
       <c r="AT3" s="0">
-        <v>13.121545504724885</v>
+        <v>45.778341320191096</v>
       </c>
       <c r="AU3" s="0">
-        <v>13.121545504724885</v>
+        <v>45.778341320191096</v>
       </c>
       <c r="AV3" s="0">
         <v>0</v>
       </c>
       <c r="AW3" s="0">
-        <v>4.4042628586591466</v>
+        <v>4.9605791270193826</v>
       </c>
       <c r="AX3" s="0">
-        <v>3.9394380249465066</v>
+        <v>4.9693449422630653</v>
       </c>
       <c r="AY3" s="0">
-        <v>3.9394380249465066</v>
+        <v>4.9693449422630653</v>
       </c>
       <c r="AZ3" s="0">
         <v>0</v>
       </c>
       <c r="BA3" s="0">
-        <v>0.096626270352799248</v>
+        <v>0.11398524614618244</v>
       </c>
       <c r="BB3" s="0">
-        <v>0.10125757242351641</v>
+        <v>0.11991779112556344</v>
       </c>
       <c r="BC3" s="0">
-        <v>0.10125757242351641</v>
+        <v>0.11991779112556344</v>
       </c>
     </row>
     <row r="4">
@@ -816,7 +816,7 @@
         <v>9.9999999999999995e-08</v>
       </c>
       <c r="F4" s="0">
-        <v>0.001</v>
+        <v>0.00050000000000000001</v>
       </c>
       <c r="G4" s="0">
         <v>5</v>
@@ -828,142 +828,142 @@
         <v>456.72653958944289</v>
       </c>
       <c r="J4" s="0">
-        <v>540.20486815260654</v>
+        <v>621.94971594098104</v>
       </c>
       <c r="K4" s="0">
-        <v>549.89140858672499</v>
+        <v>623.78802580871377</v>
       </c>
       <c r="L4" s="0">
-        <v>549.89140858672499</v>
+        <v>623.78802580871377</v>
       </c>
       <c r="M4" s="0">
         <v>-32.676170186531131</v>
       </c>
       <c r="N4" s="0">
-        <v>-30.951141600791221</v>
+        <v>-24.718937424899057</v>
       </c>
       <c r="O4" s="0">
-        <v>-30.433364581043254</v>
+        <v>-24.297892635989349</v>
       </c>
       <c r="P4" s="0">
-        <v>-30.433364581043254</v>
+        <v>-24.297892635989349</v>
       </c>
       <c r="Q4" s="0">
         <v>0.85109775601218884</v>
       </c>
       <c r="R4" s="0">
-        <v>1.0146928311762144</v>
+        <v>1.0845880660396914</v>
       </c>
       <c r="S4" s="0">
-        <v>1.0264096419169355</v>
+        <v>1.0888466791820974</v>
       </c>
       <c r="T4" s="0">
-        <v>1.0264096419169355</v>
+        <v>1.0888466791820974</v>
       </c>
       <c r="U4" s="0">
         <v>1</v>
       </c>
       <c r="V4" s="0">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="W4" s="0">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="X4" s="0">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Y4" s="0">
         <v>0</v>
       </c>
       <c r="Z4" s="0">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AA4" s="0">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AB4" s="0">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AC4" s="0">
         <v>0</v>
       </c>
       <c r="AD4" s="0">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AE4" s="0">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="AF4" s="0">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="AG4" s="0">
         <v>100</v>
       </c>
       <c r="AH4" s="0">
-        <v>95.606694560669453</v>
+        <v>94.735006973500703</v>
       </c>
       <c r="AI4" s="0">
-        <v>95.606694560669453</v>
+        <v>94.735006973500703</v>
       </c>
       <c r="AJ4" s="0">
-        <v>95.606694560669453</v>
+        <v>94.735006973500703</v>
       </c>
       <c r="AK4" s="0">
-        <v>95.404463040446302</v>
+        <v>94.548465829846577</v>
       </c>
       <c r="AL4" s="0">
-        <v>95.404463040446302</v>
+        <v>94.548465829846577</v>
       </c>
       <c r="AM4" s="0">
-        <v>15.199999999999999</v>
+        <v>18.5</v>
       </c>
       <c r="AN4" s="0">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="AO4" s="0">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="AP4" s="0">
         <v>1</v>
       </c>
       <c r="AQ4" s="0">
-        <v>0.018234865061998541</v>
+        <v>0.02401545822598454</v>
       </c>
       <c r="AR4" s="0">
         <v>0</v>
       </c>
       <c r="AS4" s="0">
-        <v>83.478328563163643</v>
+        <v>165.22317635153811</v>
       </c>
       <c r="AT4" s="0">
-        <v>93.164868997282113</v>
+        <v>167.06148621927088</v>
       </c>
       <c r="AU4" s="0">
-        <v>93.164868997282113</v>
+        <v>167.06148621927088</v>
       </c>
       <c r="AV4" s="0">
         <v>0</v>
       </c>
       <c r="AW4" s="0">
-        <v>1.7250285857399072</v>
+        <v>7.9572327616320715</v>
       </c>
       <c r="AX4" s="0">
-        <v>2.2428056054878742</v>
+        <v>8.3782775505417799</v>
       </c>
       <c r="AY4" s="0">
-        <v>2.2428056054878742</v>
+        <v>8.3782775505417799</v>
       </c>
       <c r="AZ4" s="0">
         <v>0</v>
       </c>
       <c r="BA4" s="0">
-        <v>0.16359507516402561</v>
+        <v>0.23349031002750253</v>
       </c>
       <c r="BB4" s="0">
-        <v>0.17531188590474667</v>
+        <v>0.23774892316990859</v>
       </c>
       <c r="BC4" s="0">
-        <v>0.17531188590474667</v>
+        <v>0.23774892316990859</v>
       </c>
     </row>
   </sheetData>

</xml_diff>